<commit_message>
docs(sprint 5): update sprint 4, création sprint 5(backlog)
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-sprint-backlog-v4.0.xlsx
+++ b/docs/cadrage/equipe-09-sprint-backlog-v4.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" state="visible" r:id="rId3"/>
@@ -18,7 +18,9 @@
     <sheet name="Burndown Sprint 3" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Sprint 4" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="Burndown Sprint 4" sheetId="10" state="visible" r:id="rId12"/>
-    <sheet name="Auto-évaluation" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Sprint 5" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Burndown Sprint 5" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Auto-évaluation" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="280">
   <si>
     <t xml:space="preserve">A</t>
   </si>
@@ -71,19 +73,19 @@
     <t xml:space="preserve">Sprint concerné</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 4</t>
+    <t xml:space="preserve">Sprint 5</t>
   </si>
   <si>
     <t xml:space="preserve">Version</t>
   </si>
   <si>
-    <t xml:space="preserve">V4.0</t>
+    <t xml:space="preserve">V5.0</t>
   </si>
   <si>
     <t xml:space="preserve">Date de remise</t>
   </si>
   <si>
-    <t xml:space="preserve">01/07/2026 13h00</t>
+    <t xml:space="preserve">01/07/2026 18h00</t>
   </si>
   <si>
     <t xml:space="preserve">Statut</t>
@@ -634,19 +636,14 @@
     <t xml:space="preserve">SPRINT BACKLOG : SPRINT 4</t>
   </si>
   <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mercredi 31/07/2026, 9h00 à 13h00 (4 h)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF1E1B4B"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">sécurisation prompt injection (perturbation J3)+ Conformité RGPD SAR (J3-bis) 
+    <t xml:space="preserve">sécurisation prompt injection (perturbation J3)+ Conformité RGPD SAR (J3-bis) 
 </t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">US-24</t>
@@ -658,79 +655,160 @@
     <t xml:space="preserve">Jeu ≥ 5 tests adversariaux pytest (clair, blanc-sur-blanc, langue, base64, unicode) + doc avant/après patch</t>
   </si>
   <si>
+    <t xml:space="preserve">T-24.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patch llm/ : séparation system/user (messages structurés) + instruction défensive + validation post-LLM (4 options + 1 correcte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-24.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note sécurité 1 page docs/ (diagnostic / stratégie / limites résiduelles)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-24.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 1 test adversarial automatisé dans GitHub Actions CI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-24.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérifier CA-J3-7 : les 5 tests adversariaux passent après patch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-12.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint GET /api/accounts/me/export/ — JSON structuré filtré strictement par request.user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-12.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second format export (CSV ou ZIP : quizz.json + reponses.csv + audit.json) + Content-Disposition: attachment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-12.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bouton « Exporter mes données » page profil + téléchargement automatique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-12.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modèle DataRequest (audit trail SAR) + politique de rétention 1 page docs/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-12.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réponse écrite Hugo Petit + tests pytest anti-fuite inter-comptes (user A ≠ données user B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURNDOWN : SPRINT 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09h00, Début sprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10h00, Daily intermédiaire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11h00, Mi-sprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12h00, Avant clôture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13h00, Fin sprint / Review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPRINT BACKLOG : SPRINT 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mercredi 31/07/2026, 13h00 à 18h00 (4 h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difficulté + historique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endpoint GET /api/courses/ — liste paginée filtrée request.user</t>
+  </si>
+  <si>
     <t xml:space="preserve">Todo</t>
   </si>
   <si>
-    <t xml:space="preserve">T-24.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patch llm/ : séparation system/user (messages structurés) + instruction défensive + validation post-LLM (4 options + 1 correcte)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-24.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note sécurité 1 page docs/ (diagnostic / stratégie / limites résiduelles)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-24.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥ 1 test adversarial automatisé dans GitHub Actions CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-24.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vérifier CA-J3-7 : les 5 tests adversariaux passent après patch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-12.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endpoint GET /api/accounts/me/export/ — JSON structuré filtré strictement par request.user</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-12.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Second format export (CSV ou ZIP : quizz.json + reponses.csv + audit.json) + Content-Disposition: attachment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-12.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bouton « Exporter mes données » page profil + téléchargement automatique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-12.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modèle DataRequest (audit trail SAR) + politique de rétention 1 page docs/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-12.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réponse écrite Hugo Petit + tests pytest anti-fuite inter-comptes (user A ≠ données user B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09h00, Début sprint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10h00, Daily intermédiaire</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11h00, Mi-sprint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12h00, Avant clôture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13h00, Fin sprint / Review</t>
+    <t xml:space="preserve">T-08.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serializer + annotate nb_quizz + tests API</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page frontend /library + empty state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route /library + lien nav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-08.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests pytest anti-fuite + vitest LibraryPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST /api/quizzes/generate/ — difficulty + nb_questions (5-20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patch quiz_prompt.py — 3 niveaux + nb variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI difficulté + slider 5-20 sur GenerateQuizPage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests pytest génération (bornes + niveaux)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-09.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note doc critères CA US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BURNDOWN : SPRINT 5</t>
   </si>
   <si>
     <t xml:space="preserve">✅ Grille d'auto-évaluation</t>
@@ -806,7 +884,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1034,9 +1112,16 @@
       <color rgb="FF1E1B4B"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1100,7 +1185,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE994"/>
-        <bgColor rgb="FFDDE8CB"/>
+        <bgColor rgb="FFFFF5CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -1113,6 +1198,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFDDE8CB"/>
         <bgColor rgb="FFDEE6EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD7D7"/>
+        <bgColor rgb="FFDEE6EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF5CE"/>
+        <bgColor rgb="FFFFFFD7"/>
       </patternFill>
     </fill>
   </fills>
@@ -1180,228 +1277,240 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1421,7 +1530,7 @@
       <rgbColor rgb="FFDC2626"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFD4EA6B"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
@@ -1442,7 +1551,7 @@
       <rgbColor rgb="FFE0C2CD"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFFF5CE"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
@@ -1455,7 +1564,7 @@
       <rgbColor rgb="FFDEE6EF"/>
       <rgbColor rgb="FFFFFBEB"/>
       <rgbColor rgb="FFF8FAFC"/>
-      <rgbColor rgb="FFD4EA6B"/>
+      <rgbColor rgb="FFFFD7D7"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1726,7 +1835,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>198</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1767,65 +1876,85 @@
     </row>
     <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B8" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
+      <c r="C8" s="39" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" s="19" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
+      <c r="C9" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" s="19" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
+      <c r="C10" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" s="39" t="n">
+        <v>2</v>
+      </c>
       <c r="E10" s="19" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="38" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B11" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
+      <c r="C11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" s="39" t="n">
+        <v>5</v>
+      </c>
       <c r="E11" s="19" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="38" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B12" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
+      <c r="C12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="39" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" s="19" t="s">
         <v>110</v>
       </c>
@@ -1891,6 +2020,628 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G1048576"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="54" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B20" s="55" t="s">
+        <v>235</v>
+      </c>
+      <c r="C20" s="55" t="s">
+        <v>236</v>
+      </c>
+      <c r="D20" s="55" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B21" s="55" t="s">
+        <v>238</v>
+      </c>
+      <c r="C21" s="55" t="s">
+        <v>239</v>
+      </c>
+      <c r="D21" s="55" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B22" s="55" t="s">
+        <v>240</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>241</v>
+      </c>
+      <c r="D22" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B23" s="55" t="s">
+        <v>242</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>243</v>
+      </c>
+      <c r="D23" s="55" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="42.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="55" t="s">
+        <v>234</v>
+      </c>
+      <c r="B24" s="55" t="s">
+        <v>244</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>245</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>67</v>
+      </c>
+      <c r="E24" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="55" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B25" s="56" t="s">
+        <v>247</v>
+      </c>
+      <c r="C25" s="56" t="s">
+        <v>248</v>
+      </c>
+      <c r="D25" s="56" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="56" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B26" s="56" t="s">
+        <v>249</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>250</v>
+      </c>
+      <c r="D26" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="56" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B27" s="56" t="s">
+        <v>251</v>
+      </c>
+      <c r="C27" s="56" t="s">
+        <v>252</v>
+      </c>
+      <c r="D27" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="56" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B28" s="56" t="s">
+        <v>253</v>
+      </c>
+      <c r="C28" s="56" t="s">
+        <v>254</v>
+      </c>
+      <c r="D28" s="56" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="56" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="56" t="s">
+        <v>246</v>
+      </c>
+      <c r="B29" s="56" t="s">
+        <v>255</v>
+      </c>
+      <c r="C29" s="56" t="s">
+        <v>256</v>
+      </c>
+      <c r="D29" s="56" t="s">
+        <v>141</v>
+      </c>
+      <c r="E29" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="56" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" s="34"/>
+      <c r="C30" s="35"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="F30" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="G30" s="34"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="1048572" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="35"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="39" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="19" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="19" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A2:D15"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1902,126 +2653,126 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
-        <v>230</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>231</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="23"/>
       <c r="B5" s="23" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>234</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="54" t="s">
-        <v>235</v>
-      </c>
-      <c r="C6" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D6" s="54" t="s">
-        <v>237</v>
+      <c r="B6" s="57" t="s">
+        <v>263</v>
+      </c>
+      <c r="C6" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D6" s="57" t="s">
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="54" t="s">
-        <v>238</v>
-      </c>
-      <c r="C7" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D7" s="54" t="s">
-        <v>239</v>
+      <c r="B7" s="57" t="s">
+        <v>266</v>
+      </c>
+      <c r="C7" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D7" s="57" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="54" t="s">
-        <v>240</v>
-      </c>
-      <c r="C8" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D8" s="54" t="s">
-        <v>241</v>
+      <c r="B8" s="57" t="s">
+        <v>268</v>
+      </c>
+      <c r="C8" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D8" s="57" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="54" t="s">
-        <v>242</v>
-      </c>
-      <c r="C9" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D9" s="54" t="s">
-        <v>243</v>
+      <c r="B9" s="57" t="s">
+        <v>270</v>
+      </c>
+      <c r="C9" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D9" s="57" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="54" t="s">
-        <v>244</v>
-      </c>
-      <c r="C10" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D10" s="54"/>
+      <c r="B10" s="57" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D10" s="57"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="54" t="s">
-        <v>245</v>
-      </c>
-      <c r="C11" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D11" s="54" t="s">
-        <v>246</v>
+      <c r="B11" s="57" t="s">
+        <v>273</v>
+      </c>
+      <c r="C11" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D11" s="57" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="54" t="s">
-        <v>247</v>
-      </c>
-      <c r="C12" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D12" s="54"/>
+      <c r="B12" s="57" t="s">
+        <v>275</v>
+      </c>
+      <c r="C12" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D12" s="57"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="54" t="s">
-        <v>248</v>
-      </c>
-      <c r="C13" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D13" s="54"/>
+      <c r="B13" s="57" t="s">
+        <v>276</v>
+      </c>
+      <c r="C13" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D13" s="57"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="54" t="s">
-        <v>249</v>
-      </c>
-      <c r="C14" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D14" s="54"/>
+      <c r="B14" s="57" t="s">
+        <v>277</v>
+      </c>
+      <c r="C14" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D14" s="57"/>
     </row>
     <row r="15" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="54" t="s">
-        <v>250</v>
-      </c>
-      <c r="C15" s="55" t="s">
-        <v>236</v>
-      </c>
-      <c r="D15" s="54" t="s">
-        <v>251</v>
+      <c r="B15" s="57" t="s">
+        <v>278</v>
+      </c>
+      <c r="C15" s="58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D15" s="57" t="s">
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -4164,7 +4915,7 @@
         <v>25</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>13</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4172,7 +4923,7 @@
         <v>27</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4204,7 +4955,7 @@
         <v>35</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4280,13 +5031,13 @@
     </row>
     <row r="20" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B20" s="52" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C20" s="52" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D20" s="52" t="s">
         <v>58</v>
@@ -4298,12 +5049,12 @@
         <v>2</v>
       </c>
       <c r="G20" s="52" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="55.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B21" s="52" t="s">
         <v>206</v>
@@ -4321,12 +5072,12 @@
         <v>2</v>
       </c>
       <c r="G21" s="52" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B22" s="52" t="s">
         <v>208</v>
@@ -4344,12 +5095,12 @@
         <v>1</v>
       </c>
       <c r="G22" s="52" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B23" s="52" t="s">
         <v>210</v>
@@ -4367,12 +5118,12 @@
         <v>1</v>
       </c>
       <c r="G23" s="52" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="42.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B24" s="52" t="s">
         <v>212</v>
@@ -4390,7 +5141,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="52" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="40.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4413,7 +5164,7 @@
         <v>2</v>
       </c>
       <c r="G25" s="53" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="41.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4436,7 +5187,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="53" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4459,7 +5210,7 @@
         <v>2</v>
       </c>
       <c r="G27" s="53" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4482,7 +5233,7 @@
         <v>2</v>
       </c>
       <c r="G28" s="53" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4505,7 +5256,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="53" t="s">
-        <v>205</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>